<commit_message>
allow rollback to filled xlsx
</commit_message>
<xml_diff>
--- a/res/OffersCustomer.xlsx
+++ b/res/OffersCustomer.xlsx
@@ -1,37 +1,66 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr/>
-  <workbookProtection/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Github\msword-properties-generator\res\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4A4DB63-9E8F-4CCF-A0E1-ED35B24EE18D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView xWindow="9756" yWindow="3816" windowWidth="28608" windowHeight="19200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="new" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="new" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+  <si>
+    <t>Klant Naam</t>
+  </si>
+  <si>
+    <t>Klant JobTitle</t>
+  </si>
+  <si>
+    <t>Klant JobReference</t>
+  </si>
+  <si>
+    <t>BMW Financial Services</t>
+  </si>
+  <si>
+    <t>Agile Master Pro</t>
+  </si>
+  <si>
+    <t>AMP-BMW-FS</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
-      <color theme="1"/>
-      <sz val="11"/>
       <scheme val="minor"/>
     </font>
     <font>
-      <b val="1"/>
+      <b/>
+      <sz val="11"/>
+      <name val="Calibri"/>
     </font>
   </fonts>
   <fills count="2">
     <fill>
-      <patternFill/>
+      <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
@@ -46,93 +75,43 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
-  <colors>
-    <indexedColors>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00000000"/>
-      <rgbColor rgb="00FFFFFF"/>
-      <rgbColor rgb="00FF0000"/>
-      <rgbColor rgb="0000FF00"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008000"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00808000"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="00C0C0C0"/>
-      <rgbColor rgb="00808080"/>
-      <rgbColor rgb="009999FF"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00FFFFCC"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00660066"/>
-      <rgbColor rgb="00FF8080"/>
-      <rgbColor rgb="000066CC"/>
-      <rgbColor rgb="00CCCCFF"/>
-      <rgbColor rgb="00000080"/>
-      <rgbColor rgb="00FF00FF"/>
-      <rgbColor rgb="00FFFF00"/>
-      <rgbColor rgb="0000FFFF"/>
-      <rgbColor rgb="00800080"/>
-      <rgbColor rgb="00800000"/>
-      <rgbColor rgb="00008080"/>
-      <rgbColor rgb="000000FF"/>
-      <rgbColor rgb="0000CCFF"/>
-      <rgbColor rgb="00CCFFFF"/>
-      <rgbColor rgb="00CCFFCC"/>
-      <rgbColor rgb="00FFFF99"/>
-      <rgbColor rgb="0099CCFF"/>
-      <rgbColor rgb="00FF99CC"/>
-      <rgbColor rgb="00CC99FF"/>
-      <rgbColor rgb="00FFCC99"/>
-      <rgbColor rgb="003366FF"/>
-      <rgbColor rgb="0033CCCC"/>
-      <rgbColor rgb="0099CC00"/>
-      <rgbColor rgb="00FFCC00"/>
-      <rgbColor rgb="00FF9900"/>
-      <rgbColor rgb="00FF6600"/>
-      <rgbColor rgb="00666699"/>
-      <rgbColor rgb="00969696"/>
-      <rgbColor rgb="00003366"/>
-      <rgbColor rgb="00339966"/>
-      <rgbColor rgb="00003300"/>
-      <rgbColor rgb="00333300"/>
-      <rgbColor rgb="00993300"/>
-      <rgbColor rgb="00993366"/>
-      <rgbColor rgb="00333399"/>
-      <rgbColor rgb="00333333"/>
-    </indexedColors>
-  </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
@@ -420,29 +399,35 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:C2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="20.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.33203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Klant Naam</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Klant JobTitle</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Klant JobReference</t>
-        </is>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
new commit as trigger actions
</commit_message>
<xml_diff>
--- a/res/OffersCustomer.xlsx
+++ b/res/OffersCustomer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Github\msword-properties-generator\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{47C125E8-34F9-46EA-9723-CE774CF39B02}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FFF56F59-7C1E-4D8B-9E2C-C6D153CB1CCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9756" yWindow="3816" windowWidth="28608" windowHeight="19200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Klant Naam</t>
   </si>
@@ -29,15 +29,6 @@
   </si>
   <si>
     <t>Klant JobReference</t>
-  </si>
-  <si>
-    <t>BMW Financial Services</t>
-  </si>
-  <si>
-    <t>Agile Master Pro</t>
-  </si>
-  <si>
-    <t>AMP-BMW-FS</t>
   </si>
   <si>
     <t>Fluvius SA</t>
@@ -409,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.33203125" bestFit="1" customWidth="1"/>
@@ -439,17 +430,6 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>6</v>
-      </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" t="s">
-        <v>8</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
trigger to actions again
</commit_message>
<xml_diff>
--- a/res/OffersCustomer.xlsx
+++ b/res/OffersCustomer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Github\msword-properties-generator\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{485E116F-F55D-4D43-B4F7-72017D3A3CCA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A319B104-32D9-4F1D-9BAF-FD8AE946DA9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9756" yWindow="3816" windowWidth="28608" windowHeight="19200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
     <t>Senior Scrum Master</t>
   </si>
   <si>
-    <t>FLU-SSM-ULTRA</t>
+    <t>FLU-SSM-ULTRA-PACK</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
commit & push to trigger pipeline
</commit_message>
<xml_diff>
--- a/res/OffersCustomer.xlsx
+++ b/res/OffersCustomer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Github\msword-properties-generator\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A319B104-32D9-4F1D-9BAF-FD8AE946DA9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DAF803A-18DE-4756-8DF8-E2E370F29AE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9756" yWindow="3816" windowWidth="28608" windowHeight="19200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
     <t>Senior Scrum Master</t>
   </si>
   <si>
-    <t>FLU-SSM-ULTRA-PACK</t>
+    <t>FLU-SSM-ULTRA-PACK-DICK</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
cleanup logging code + trigger new mail after push
</commit_message>
<xml_diff>
--- a/res/OffersCustomer.xlsx
+++ b/res/OffersCustomer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Github\msword-properties-generator\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DAF803A-18DE-4756-8DF8-E2E370F29AE4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31E9A126-8643-4DFA-AD89-FE2DF65AA48A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9756" yWindow="3816" windowWidth="28608" windowHeight="19200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
     <t>Senior Scrum Master</t>
   </si>
   <si>
-    <t>FLU-SSM-ULTRA-PACK-DICK</t>
+    <t>FLU-SSM-ULTRA</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
trigger test after Push
</commit_message>
<xml_diff>
--- a/res/OffersCustomer.xlsx
+++ b/res/OffersCustomer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Github\msword-properties-generator\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{31E9A126-8643-4DFA-AD89-FE2DF65AA48A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAAC3FE9-022F-4EDD-950A-45AA0BC16A8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9756" yWindow="3816" windowWidth="28608" windowHeight="19200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
   <si>
     <t>Klant Naam</t>
   </si>
@@ -38,6 +38,15 @@
   </si>
   <si>
     <t>FLU-SSM-ULTRA</t>
+  </si>
+  <si>
+    <t>BMW Fincancial Services</t>
+  </si>
+  <si>
+    <t>Agile Master</t>
+  </si>
+  <si>
+    <t>BMW-FS-AM</t>
   </si>
 </sst>
 </file>
@@ -400,7 +409,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.33203125" bestFit="1" customWidth="1"/>
@@ -430,6 +439,17 @@
         <v>5</v>
       </c>
     </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C3" t="s">
+        <v>8</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
forgot DROPBOX_TOKEN to add to env var's
</commit_message>
<xml_diff>
--- a/res/OffersCustomer.xlsx
+++ b/res/OffersCustomer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Github\msword-properties-generator\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DAAC3FE9-022F-4EDD-950A-45AA0BC16A8D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B31053A7-1836-480C-A2F4-47FA7FAB0A20}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="9756" yWindow="3816" windowWidth="28608" windowHeight="19200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -43,10 +43,10 @@
     <t>BMW Fincancial Services</t>
   </si>
   <si>
-    <t>Agile Master</t>
-  </si>
-  <si>
-    <t>BMW-FS-AM</t>
+    <t>Agile Master HYPER</t>
+  </si>
+  <si>
+    <t>BMW-FS-AMHYPER</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
trigger test when xlsx is pushed
</commit_message>
<xml_diff>
--- a/res/OffersCustomer.xlsx
+++ b/res/OffersCustomer.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Github\msword-properties-generator\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{08A8BC68-AB81-496E-935D-5DEA4F6C592F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAED5E31-9DF6-4299-A914-7863C383044F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="9756" yWindow="3816" windowWidth="28608" windowHeight="19200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2556" yWindow="6000" windowWidth="28608" windowHeight="19200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="new" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Klant Naam</t>
   </si>
@@ -31,22 +31,13 @@
     <t>Klant JobReference</t>
   </si>
   <si>
-    <t>Fluvius SA</t>
-  </si>
-  <si>
-    <t>BMW Fincancial Services</t>
-  </si>
-  <si>
-    <t>Junior Scrum Master</t>
-  </si>
-  <si>
-    <t>FLU-SSM-JUNIOR</t>
-  </si>
-  <si>
-    <t>Junior Agile Master</t>
-  </si>
-  <si>
-    <t>BMW-FS</t>
+    <t>Vlaamse Radio en Televisie omroep (VRT)</t>
+  </si>
+  <si>
+    <t>Scrum Master Dataplatform</t>
+  </si>
+  <si>
+    <t>VRT-SMDP-002</t>
   </si>
 </sst>
 </file>
@@ -409,11 +400,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.33203125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.77734375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="17.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -433,21 +424,10 @@
         <v>3</v>
       </c>
       <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
         <v>5</v>
-      </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>4</v>
-      </c>
-      <c r="B3" t="s">
-        <v>7</v>
-      </c>
-      <c r="C3" t="s">
-        <v>8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
trigger test when xlsx is pushed + not mandatory fields
</commit_message>
<xml_diff>
--- a/res/OffersCustomer.xlsx
+++ b/res/OffersCustomer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Github\msword-properties-generator\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CAED5E31-9DF6-4299-A914-7863C383044F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BE886B0-C906-48CF-BC24-0198AF91466E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2556" yWindow="6000" windowWidth="28608" windowHeight="19200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
     <t>Scrum Master Dataplatform</t>
   </si>
   <si>
-    <t>VRT-SMDP-002</t>
+    <t>VRT-SMDP-003</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
trigger test when xlsx is pushed while other pipeline is running
</commit_message>
<xml_diff>
--- a/res/OffersCustomer.xlsx
+++ b/res/OffersCustomer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Github\msword-properties-generator\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0BE886B0-C906-48CF-BC24-0198AF91466E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{590FEE00-71AD-4682-BA07-9EDAF6B2483D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2556" yWindow="6000" windowWidth="28608" windowHeight="19200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
     <t>Scrum Master Dataplatform</t>
   </si>
   <si>
-    <t>VRT-SMDP-003</t>
+    <t>VRT-SMDP-004</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
caching strategies to speed up pipeline fixes
</commit_message>
<xml_diff>
--- a/res/OffersCustomer.xlsx
+++ b/res/OffersCustomer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Github\msword-properties-generator\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2CDB3C1C-4400-4474-82A1-8705FEE0725B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B19A77A3-C61A-4207-B4DE-B89BF6B505CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2556" yWindow="6000" windowWidth="28608" windowHeight="19200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
     <t>Scrum Master Dataplatform</t>
   </si>
   <si>
-    <t>VRT-SMDP-005</t>
+    <t>VRT-SMDP-006</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
List cache content on several moments
</commit_message>
<xml_diff>
--- a/res/OffersCustomer.xlsx
+++ b/res/OffersCustomer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Github\msword-properties-generator\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EDB6A4F9-4D8E-4908-81F7-4C0F9C7EF5FD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4F4B24A-D364-47DD-9961-BAB7F8D42DAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2556" yWindow="6000" windowWidth="28608" windowHeight="19200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
     <t>Scrum Master Dataplatform</t>
   </si>
   <si>
-    <t>VRT-SMDP-019</t>
+    <t>VRT-SMDP-020</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Learn about caching, listing it all
</commit_message>
<xml_diff>
--- a/res/OffersCustomer.xlsx
+++ b/res/OffersCustomer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Github\msword-properties-generator\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C4F4B24A-D364-47DD-9961-BAB7F8D42DAC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F1D67EFA-5F0B-4E51-8A42-A467AE943D3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2556" yWindow="6000" windowWidth="28608" windowHeight="19200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
     <t>Scrum Master Dataplatform</t>
   </si>
   <si>
-    <t>VRT-SMDP-020</t>
+    <t>VRT-SMDP-021</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Cleaning Extractions & show all Cache keys consistently
</commit_message>
<xml_diff>
--- a/res/OffersCustomer.xlsx
+++ b/res/OffersCustomer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Github\msword-properties-generator\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ACFEB203-0A49-4D17-997D-2A15477FC1C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69D21F72-EB84-4665-97E5-040044E8B71C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2556" yWindow="6000" windowWidth="28608" windowHeight="19200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
     <t>Scrum Master Dataplatform</t>
   </si>
   <si>
-    <t>VRT-SMDP-022</t>
+    <t>VRT-SMDP-023</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Order of stuff consistently; Pip, Jdk, LibreOffice
</commit_message>
<xml_diff>
--- a/res/OffersCustomer.xlsx
+++ b/res/OffersCustomer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Github\msword-properties-generator\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{69D21F72-EB84-4665-97E5-040044E8B71C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB8CC9C5-2A22-4EED-81F9-48E9F1E72ECB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2556" yWindow="6000" windowWidth="28608" windowHeight="19200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
     <t>Scrum Master Dataplatform</t>
   </si>
   <si>
-    <t>VRT-SMDP-023</t>
+    <t>VRT-SMDP-024</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
Dropbox long-term access guaranteed
</commit_message>
<xml_diff>
--- a/res/OffersCustomer.xlsx
+++ b/res/OffersCustomer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Github\msword-properties-generator\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB8CC9C5-2A22-4EED-81F9-48E9F1E72ECB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{247AB6BE-C6CB-44F4-9E48-8943EADCC413}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2556" yWindow="6000" windowWidth="28608" windowHeight="19200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
     <t>Scrum Master Dataplatform</t>
   </si>
   <si>
-    <t>VRT-SMDP-024</t>
+    <t>VRT-SMDP-025</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
We can clean this up now.
</commit_message>
<xml_diff>
--- a/res/OffersCustomer.xlsx
+++ b/res/OffersCustomer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Github\msword-properties-generator\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0801AA4C-2009-4588-BD73-93737E60F0A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B2A77B6-EC91-47D6-A0E5-2B89E0FCF26C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2556" yWindow="6000" windowWidth="28608" windowHeight="19200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
   <si>
     <t>Klant Naam</t>
   </si>
@@ -29,15 +29,6 @@
   </si>
   <si>
     <t>Klant JobReference</t>
-  </si>
-  <si>
-    <t>Vlaamse Radio en Televisie omroep (VRT)</t>
-  </si>
-  <si>
-    <t>Scrum Master Dataplatform</t>
-  </si>
-  <si>
-    <t>VRT-SMDP-026</t>
   </si>
 </sst>
 </file>
@@ -400,7 +391,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.33203125" bestFit="1" customWidth="1"/>
@@ -419,17 +410,6 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C2" t="s">
-        <v>5</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
testing pipeline with all local working tests
</commit_message>
<xml_diff>
--- a/res/OffersCustomer.xlsx
+++ b/res/OffersCustomer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Github\msword-properties-generator\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B2A77B6-EC91-47D6-A0E5-2B89E0FCF26C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{80651C8E-0046-4312-808E-0D99F733438D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2556" yWindow="6000" windowWidth="28608" windowHeight="19200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3" uniqueCount="3">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Klant Naam</t>
   </si>
@@ -29,6 +29,15 @@
   </si>
   <si>
     <t>Klant JobReference</t>
+  </si>
+  <si>
+    <t>BMW Financial Services</t>
+  </si>
+  <si>
+    <t>Agile Master Senior</t>
+  </si>
+  <si>
+    <t>BMW-FS-AMS006</t>
   </si>
 </sst>
 </file>
@@ -391,7 +400,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20.33203125" bestFit="1" customWidth="1"/>
@@ -410,6 +419,17 @@
         <v>2</v>
       </c>
     </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>3</v>
+      </c>
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C2" t="s">
+        <v>5</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Added the non-manual workflow_dispatch to avoid skipping on: Push + trigger on: Push to test
</commit_message>
<xml_diff>
--- a/res/OffersCustomer.xlsx
+++ b/res/OffersCustomer.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projects\Github\msword-properties-generator\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F14F2B35-3BCC-4112-8900-CC32CFD8D1F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD58F45F-BD01-4D04-990F-AA6ADC5D9485}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2556" yWindow="6000" windowWidth="28608" windowHeight="19200" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
     <t>Agile Master Senior</t>
   </si>
   <si>
-    <t>BMW-FS-AMS008</t>
+    <t>BMW-FS-AMS009</t>
   </si>
 </sst>
 </file>

</xml_diff>